<commit_message>
Atualizacao do sistema de vistoria de sedes
</commit_message>
<xml_diff>
--- a/relatorios e formularios/Visitas_Monitoramento_Sedes_Kobo.xlsx
+++ b/relatorios e formularios/Visitas_Monitoramento_Sedes_Kobo.xlsx
@@ -3907,7 +3907,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -4179,7 +4179,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -4545,7 +4545,7 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -5085,7 +5085,7 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -5289,7 +5289,7 @@
         </is>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -5561,7 +5561,7 @@
         </is>
       </c>
       <c r="M23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -5659,7 +5659,7 @@
         </is>
       </c>
       <c r="M24" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -5761,7 +5761,7 @@
         </is>
       </c>
       <c r="M25" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -5931,7 +5931,7 @@
         </is>
       </c>
       <c r="M27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -6169,7 +6169,7 @@
         </is>
       </c>
       <c r="M30" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -6267,11 +6267,11 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Amarelo (8 a 15 dias)</t>
+          <t>Vermelho (&gt;= 16 dias)</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -6637,7 +6637,7 @@
         </is>
       </c>
       <c r="M36" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -6943,7 +6943,7 @@
         </is>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -7181,7 +7181,7 @@
         </is>
       </c>
       <c r="M43" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -7351,7 +7351,7 @@
         </is>
       </c>
       <c r="M45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -7793,7 +7793,7 @@
         </is>
       </c>
       <c r="M51" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -7963,7 +7963,7 @@
         </is>
       </c>
       <c r="M53" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -8129,7 +8129,7 @@
         </is>
       </c>
       <c r="M55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="M61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -8737,7 +8737,7 @@
         </is>
       </c>
       <c r="M63" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -8907,7 +8907,7 @@
         </is>
       </c>
       <c r="M65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -9281,7 +9281,7 @@
         </is>
       </c>
       <c r="M70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -9383,7 +9383,7 @@
         </is>
       </c>
       <c r="M71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -9689,7 +9689,7 @@
         </is>
       </c>
       <c r="M75" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -9927,7 +9927,7 @@
         </is>
       </c>
       <c r="M78" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>

</xml_diff>